<commit_message>
Fix action plan workbook export and seed chapter 0
</commit_message>
<xml_diff>
--- a/AutoBericht/project-template/templates/Vorlage Aktionsplan d.xlsx
+++ b/AutoBericht/project-template/templates/Vorlage Aktionsplan d.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent>
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -118,7 +118,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -137,6 +137,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -150,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -177,6 +183,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -754,11 +761,11 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <ns3:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <ns4:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1135,7 +1142,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T9"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1202,8 +1209,16 @@
       <c r="T2" s="7"/>
     </row>
     <row r="3" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aktualisiert am</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -1880,9 +1895,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
+  <mergeCells count="3">
     <mergeCell ref="J3:L3"/>
     <mergeCell ref="M3:P3"/>
     <mergeCell ref="Q3:T3"/>

</xml_diff>